<commit_message>
Fix no date shift upload
</commit_message>
<xml_diff>
--- a/staffsync-shift-upload-template.xlsx
+++ b/staffsync-shift-upload-template.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Shift Upload" sheetId="1" r:id="R476cd2f657eb418b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="2" r:id="R5259fe1f0deb4156"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Shift Upload" sheetId="1" r:id="R6152b4778e6a4765"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="2" r:id="R6d058f73f4464fbd"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -14,9 +14,6 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="1">
-    <x:numFmt numFmtId="200" formatCode="yyyy-mm-dd"/>
-  </x:numFmts>
   <x:fonts count="4">
     <x:font>
       <x:sz val="11"/>
@@ -78,7 +75,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="12">
+  <x:cellXfs count="11">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -89,9 +86,6 @@
       <x:alignment wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="200" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment wrapText="1"/>
-    </x:xf>
     <x:xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -316,50 +310,46 @@
     <x:col min="11" max="11" width="15" hidden="0" customWidth="1"/>
     <x:col min="12" max="12" width="15" hidden="0" customWidth="1"/>
     <x:col min="13" max="13" width="15" hidden="0" customWidth="1"/>
-    <x:col min="14" max="14" width="15" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
       <x:c r="A1" s="4" t="str">
         <x:v>employee_code</x:v>
       </x:c>
-      <x:c r="B1" s="6" t="str">
-        <x:v>date</x:v>
+      <x:c r="B1" s="4" t="str">
+        <x:v>shift</x:v>
       </x:c>
       <x:c r="C1" s="4" t="str">
-        <x:v>shift</x:v>
+        <x:v>in_time</x:v>
       </x:c>
       <x:c r="D1" s="4" t="str">
-        <x:v>in_time</x:v>
+        <x:v>out_time</x:v>
       </x:c>
       <x:c r="E1" s="4" t="str">
-        <x:v>out_time</x:v>
+        <x:v>status</x:v>
       </x:c>
       <x:c r="F1" s="4" t="str">
-        <x:v>status</x:v>
+        <x:v>shift_2</x:v>
       </x:c>
       <x:c r="G1" s="4" t="str">
-        <x:v>shift_2</x:v>
+        <x:v>in_time_2</x:v>
       </x:c>
       <x:c r="H1" s="4" t="str">
-        <x:v>in_time_2</x:v>
+        <x:v>out_time_2</x:v>
       </x:c>
       <x:c r="I1" s="4" t="str">
-        <x:v>out_time_2</x:v>
+        <x:v>status_2</x:v>
       </x:c>
       <x:c r="J1" s="4" t="str">
-        <x:v>status_2</x:v>
+        <x:v>shift_3</x:v>
       </x:c>
       <x:c r="K1" s="4" t="str">
-        <x:v>shift_3</x:v>
+        <x:v>in_time_3</x:v>
       </x:c>
       <x:c r="L1" s="4" t="str">
-        <x:v>in_time_3</x:v>
+        <x:v>out_time_3</x:v>
       </x:c>
       <x:c r="M1" s="4" t="str">
-        <x:v>out_time_3</x:v>
-      </x:c>
-      <x:c r="N1" s="4" t="str">
         <x:v>status_3</x:v>
       </x:c>
     </x:row>
@@ -368,20 +358,18 @@
         <x:v>01</x:v>
       </x:c>
       <x:c r="B2" s="5" t="str">
-        <x:v>2026-07-22</x:v>
+        <x:v>10 hours</x:v>
       </x:c>
       <x:c r="C2" s="5" t="str">
-        <x:v>10 hours</x:v>
+        <x:v>07:00</x:v>
       </x:c>
       <x:c r="D2" s="5" t="str">
-        <x:v>07:00</x:v>
+        <x:v>17:00</x:v>
       </x:c>
       <x:c r="E2" s="5" t="str">
-        <x:v>17:00</x:v>
-      </x:c>
-      <x:c r="F2" s="5" t="str">
         <x:v>Working</x:v>
       </x:c>
+      <x:c r="F2" s="5" t="str"/>
       <x:c r="G2" s="5" t="str"/>
       <x:c r="H2" s="5" t="str"/>
       <x:c r="I2" s="5" t="str"/>
@@ -389,63 +377,57 @@
       <x:c r="K2" s="5" t="str"/>
       <x:c r="L2" s="5" t="str"/>
       <x:c r="M2" s="5" t="str"/>
-      <x:c r="N2" s="5" t="str"/>
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="5" t="str">
         <x:v>02</x:v>
       </x:c>
       <x:c r="B3" s="5" t="str">
-        <x:v>2026-07-22</x:v>
+        <x:v>Morning</x:v>
       </x:c>
       <x:c r="C3" s="5" t="str">
-        <x:v>Morning</x:v>
+        <x:v>07:00</x:v>
       </x:c>
       <x:c r="D3" s="5" t="str">
-        <x:v>07:00</x:v>
+        <x:v>15:00</x:v>
       </x:c>
       <x:c r="E3" s="5" t="str">
-        <x:v>15:00</x:v>
+        <x:v>Working</x:v>
       </x:c>
       <x:c r="F3" s="5" t="str">
+        <x:v>Evening</x:v>
+      </x:c>
+      <x:c r="G3" s="5" t="str">
+        <x:v>18:00</x:v>
+      </x:c>
+      <x:c r="H3" s="5" t="str">
+        <x:v>22:00</x:v>
+      </x:c>
+      <x:c r="I3" s="5" t="str">
         <x:v>Working</x:v>
       </x:c>
-      <x:c r="G3" s="5" t="str">
-        <x:v>Evening</x:v>
-      </x:c>
-      <x:c r="H3" s="5" t="str">
-        <x:v>18:00</x:v>
-      </x:c>
-      <x:c r="I3" s="5" t="str">
-        <x:v>22:00</x:v>
-      </x:c>
-      <x:c r="J3" s="5" t="str">
-        <x:v>Working</x:v>
-      </x:c>
+      <x:c r="J3" s="5" t="str"/>
       <x:c r="K3" s="5" t="str"/>
       <x:c r="L3" s="5" t="str"/>
       <x:c r="M3" s="5" t="str"/>
-      <x:c r="N3" s="5" t="str"/>
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="5" t="str">
         <x:v>03</x:v>
       </x:c>
       <x:c r="B4" s="5" t="str">
-        <x:v>2026-07-22</x:v>
+        <x:v>Weekly off</x:v>
       </x:c>
       <x:c r="C4" s="5" t="str">
-        <x:v>Weekly off</x:v>
+        <x:v>00:00</x:v>
       </x:c>
       <x:c r="D4" s="5" t="str">
         <x:v>00:00</x:v>
       </x:c>
       <x:c r="E4" s="5" t="str">
-        <x:v>00:00</x:v>
-      </x:c>
-      <x:c r="F4" s="5" t="str">
         <x:v>Weekly off</x:v>
       </x:c>
+      <x:c r="F4" s="5" t="str"/>
       <x:c r="G4" s="5" t="str"/>
       <x:c r="H4" s="5" t="str"/>
       <x:c r="I4" s="5" t="str"/>
@@ -453,49 +435,45 @@
       <x:c r="K4" s="5" t="str"/>
       <x:c r="L4" s="5" t="str"/>
       <x:c r="M4" s="5" t="str"/>
-      <x:c r="N4" s="5" t="str"/>
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="5" t="str">
         <x:v>04</x:v>
       </x:c>
       <x:c r="B5" s="5" t="str">
-        <x:v>2026-07-22</x:v>
+        <x:v>Morning</x:v>
       </x:c>
       <x:c r="C5" s="5" t="str">
-        <x:v>Morning</x:v>
+        <x:v>07:00</x:v>
       </x:c>
       <x:c r="D5" s="5" t="str">
-        <x:v>07:00</x:v>
+        <x:v>12:00</x:v>
       </x:c>
       <x:c r="E5" s="5" t="str">
-        <x:v>12:00</x:v>
+        <x:v>Working</x:v>
       </x:c>
       <x:c r="F5" s="5" t="str">
+        <x:v>Evening</x:v>
+      </x:c>
+      <x:c r="G5" s="5" t="str">
+        <x:v>16:00</x:v>
+      </x:c>
+      <x:c r="H5" s="5" t="str">
+        <x:v>20:00</x:v>
+      </x:c>
+      <x:c r="I5" s="5" t="str">
         <x:v>Working</x:v>
       </x:c>
-      <x:c r="G5" s="5" t="str">
-        <x:v>Evening</x:v>
-      </x:c>
-      <x:c r="H5" s="5" t="str">
-        <x:v>16:00</x:v>
-      </x:c>
-      <x:c r="I5" s="5" t="str">
-        <x:v>20:00</x:v>
-      </x:c>
       <x:c r="J5" s="5" t="str">
-        <x:v>Working</x:v>
+        <x:v>Night</x:v>
       </x:c>
       <x:c r="K5" s="5" t="str">
-        <x:v>Night</x:v>
+        <x:v>22:00</x:v>
       </x:c>
       <x:c r="L5" s="5" t="str">
-        <x:v>22:00</x:v>
+        <x:v>02:00</x:v>
       </x:c>
       <x:c r="M5" s="5" t="str">
-        <x:v>02:00</x:v>
-      </x:c>
-      <x:c r="N5" s="5" t="str">
         <x:v>Working</x:v>
       </x:c>
     </x:row>
@@ -515,93 +493,81 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1">
-      <x:c r="A1" s="7" t="str">
+      <x:c r="A1" s="6" t="str">
         <x:v>StaffSync Shift Upload Instructions</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
-      <x:c r="A3" s="10" t="str">
+      <x:c r="A3" s="9" t="str">
         <x:v>Required</x:v>
       </x:c>
-      <x:c r="B3" s="11" t="str">
+      <x:c r="B3" s="10" t="str">
         <x:v>employee_code</x:v>
       </x:c>
-      <x:c r="C3" s="11" t="str">
+      <x:c r="C3" s="10" t="str">
         <x:v>Must match StaffSync employee code, for example 01, 02, 03.</x:v>
       </x:c>
-      <x:c r="D3" s="11" t="str"/>
+      <x:c r="D3" s="10" t="str"/>
     </x:row>
     <x:row r="4">
-      <x:c r="A4" s="10" t="str">
+      <x:c r="A4" s="9" t="str">
         <x:v>Required</x:v>
       </x:c>
-      <x:c r="B4" s="11" t="str">
-        <x:v>date</x:v>
-      </x:c>
-      <x:c r="C4" s="11" t="str">
-        <x:v>Use yyyy-mm-dd, for example 2026-07-22.</x:v>
-      </x:c>
-      <x:c r="D4" s="11" t="str"/>
+      <x:c r="B4" s="10" t="str">
+        <x:v>shift</x:v>
+      </x:c>
+      <x:c r="C4" s="10" t="str">
+        <x:v>Use 10 hours, Morning, Evening, Night, Weekly off, or your own shift name.</x:v>
+      </x:c>
+      <x:c r="D4" s="10" t="str"/>
     </x:row>
     <x:row r="5">
-      <x:c r="A5" s="10" t="str">
+      <x:c r="A5" s="9" t="str">
         <x:v>Required</x:v>
       </x:c>
-      <x:c r="B5" s="11" t="str">
-        <x:v>shift</x:v>
-      </x:c>
-      <x:c r="C5" s="11" t="str">
-        <x:v>Use 10 hours, Morning, Evening, Night, Weekly off, or your own shift name.</x:v>
-      </x:c>
-      <x:c r="D5" s="11" t="str"/>
+      <x:c r="B5" s="10" t="str">
+        <x:v>in_time / out_time</x:v>
+      </x:c>
+      <x:c r="C5" s="10" t="str">
+        <x:v>Use 24 hour time, for example 07:00 and 17:00.</x:v>
+      </x:c>
+      <x:c r="D5" s="10" t="str"/>
     </x:row>
     <x:row r="6">
-      <x:c r="A6" s="10" t="str">
-        <x:v>Required</x:v>
-      </x:c>
-      <x:c r="B6" s="11" t="str">
-        <x:v>in_time / out_time</x:v>
-      </x:c>
-      <x:c r="C6" s="11" t="str">
-        <x:v>Use 24 hour time, for example 07:00 and 17:00.</x:v>
-      </x:c>
-      <x:c r="D6" s="11" t="str"/>
+      <x:c r="A6" s="9" t="str">
+        <x:v>Optional</x:v>
+      </x:c>
+      <x:c r="B6" s="10" t="str">
+        <x:v>shift_2 / shift_3</x:v>
+      </x:c>
+      <x:c r="C6" s="10" t="str">
+        <x:v>Use only when the same employee works two or three shifts on the same day.</x:v>
+      </x:c>
+      <x:c r="D6" s="10" t="str"/>
     </x:row>
     <x:row r="7">
-      <x:c r="A7" s="10" t="str">
+      <x:c r="A7" s="9" t="str">
         <x:v>Optional</x:v>
       </x:c>
-      <x:c r="B7" s="11" t="str">
-        <x:v>shift_2 / shift_3</x:v>
-      </x:c>
-      <x:c r="C7" s="11" t="str">
-        <x:v>Use only when the same employee works two or three shifts on the same day.</x:v>
-      </x:c>
-      <x:c r="D7" s="11" t="str"/>
+      <x:c r="B7" s="10" t="str">
+        <x:v>status</x:v>
+      </x:c>
+      <x:c r="C7" s="10" t="str">
+        <x:v>Use Working, Extra shift, Weekly off, Leave, Half day, Short leave.</x:v>
+      </x:c>
+      <x:c r="D7" s="10" t="str"/>
     </x:row>
     <x:row r="8">
-      <x:c r="A8" s="10" t="str">
-        <x:v>Optional</x:v>
-      </x:c>
-      <x:c r="B8" s="11" t="str">
-        <x:v>status</x:v>
-      </x:c>
-      <x:c r="C8" s="11" t="str">
-        <x:v>Use Working, Extra shift, Weekly off, Leave, Half day, Short leave.</x:v>
-      </x:c>
-      <x:c r="D8" s="11" t="str"/>
-    </x:row>
-    <x:row r="9">
-      <x:c r="A9" s="10" t="str">
-        <x:v>Tip</x:v>
-      </x:c>
-      <x:c r="B9" s="11" t="str">
-        <x:v>Google Sheets</x:v>
-      </x:c>
-      <x:c r="C9" s="11" t="str">
-        <x:v>Open your Google sheet, choose File &gt; Download &gt; Microsoft Excel (.xlsx), then upload it in StaffSync.</x:v>
-      </x:c>
-      <x:c r="D9" s="11" t="str"/>
+      <x:c r="A8" s="9" t="str">
+        <x:v>Date</x:v>
+      </x:c>
+      <x:c r="B8" s="10" t="str">
+        <x:v>No date column needed</x:v>
+      </x:c>
+      <x:c r="C8" s="10" t="str">
+        <x:v>Choose the upload date inside StaffSync before clicking import.</x:v>
+      </x:c>
+      <x:c r="D8" s="10" t="str"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>

</xml_diff>